<commit_message>
updated the stemmer to be more accurate about uncategorized comments
</commit_message>
<xml_diff>
--- a/5kcategorydataset.xlsx
+++ b/5kcategorydataset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\OneDrive\Documents\Library Management System\hllsystem - Oct10-2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2D1403-3626-4479-B68B-854E17191FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B795F75B-2CE1-4F10-ADC7-AD1E31EC1778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="2640" windowWidth="18015" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Data" sheetId="1" r:id="rId1"/>
@@ -13627,7 +13627,7 @@
   <dimension ref="A1:B5001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="93.28515625" customWidth="1"/>
+    <col min="1" max="1" width="96.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>